<commit_message>
Update(ReportesCredito): Update python file to add method main to be call from the bot
</commit_message>
<xml_diff>
--- a/Archivos/CONFIGURACION/Config.xlsx
+++ b/Archivos/CONFIGURACION/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\CONFIGURACION\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Procesos_Uipath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\CONFIGURACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9A5910-4476-4BCE-96B8-2C3C6A5E8364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{803D8319-F394-45CB-9522-84A687AF6C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="235">
   <si>
     <t>Name</t>
   </si>
@@ -568,9 +568,6 @@
   </si>
   <si>
     <t>Colocar el ID principal del espacio en drive</t>
-  </si>
-  <si>
-    <t>D:\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json</t>
   </si>
   <si>
     <t>crp-pro-ccoe-automat-neg-finan@crp-pro-ccoe-automat.iam.gserviceaccount.com</t>
@@ -841,6 +838,12 @@
   </si>
   <si>
     <t>ZIP_ERROR</t>
+  </si>
+  <si>
+    <t>UBICACION</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
 </sst>
 </file>
@@ -1512,12 +1515,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z990"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="71.140625" customWidth="1"/>
+    <col min="1" max="1" width="43.54296875" customWidth="1"/>
+    <col min="2" max="2" width="71.1796875" customWidth="1"/>
     <col min="3" max="3" width="92" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1557,15 +1560,18 @@
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:26" ht="15.75">
+    <row r="3" spans="1:26" ht="15.5">
       <c r="A3" s="24" t="s">
         <v>123</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>128</v>
+      </c>
+      <c r="E3" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -1578,8 +1584,11 @@
       <c r="C4" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="5" spans="1:26">
+      <c r="E4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.5">
       <c r="A5" s="10" t="s">
         <v>46</v>
       </c>
@@ -1593,7 +1602,7 @@
         <v>132</v>
       </c>
       <c r="B6" s="2" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"</f>
+        <f>_xlfn.CONCAT(E4, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -1605,7 +1614,7 @@
         <v>47</v>
       </c>
       <c r="B7" s="2" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"\"</f>
+        <f>_xlfn.CONCAT(E4, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"\")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\Temporal\</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -1617,7 +1626,7 @@
         <v>135</v>
       </c>
       <c r="B8" s="2" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;""</f>
+        <f>_xlfn.CONCAT(E4, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\Temporal</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -1629,7 +1638,7 @@
         <v>48</v>
       </c>
       <c r="B9" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;B3&amp;"\Archivos\FORMATOS\"</f>
+        <f>_xlfn.CONCAT(E4, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\FORMATOS\")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\FORMATOS\</v>
       </c>
       <c r="C9" t="s">
@@ -1641,7 +1650,7 @@
         <v>138</v>
       </c>
       <c r="B10" s="2" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;B3&amp;"\Archivos\CONFIGURACION\"</f>
+        <f>_xlfn.CONCAT(E4, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\CONFIGURACION\")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\CONFIGURACION\</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -1653,7 +1662,7 @@
         <v>140</v>
       </c>
       <c r="B11" s="2" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;B3&amp;"\Archivos\Exceptions_Screenshots\"</f>
+        <f>_xlfn.CONCAT(E4, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\Exceptions_Screenshots\")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\Exceptions_Screenshots\</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1662,10 +1671,10 @@
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B12" s="2" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"_ERROR.zip"</f>
+        <f>_xlfn.CONCAT(E4, ":\Procesos_UiPath\"&amp;B3&amp;"\Archivos\"&amp;B4&amp;"_ERROR.zip")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\Temporal_ERROR.zip</v>
       </c>
       <c r="C12" s="2"/>
@@ -1675,15 +1684,15 @@
         <v>142</v>
       </c>
       <c r="B13" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" ht="14.1" customHeight="1">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="14.15" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>143</v>
       </c>
       <c r="B14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -1715,14 +1724,14 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" ht="14.5">
       <c r="A24" s="20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
     </row>
-    <row r="25" spans="1:3" ht="14.1" customHeight="1">
+    <row r="25" spans="1:3" ht="14.15" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -1830,7 +1839,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="14.1" customHeight="1">
+    <row r="39" spans="1:4" ht="14.15" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>155</v>
       </c>
@@ -1850,7 +1859,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="12.95" customHeight="1">
+    <row r="41" spans="1:4" ht="13" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>160</v>
       </c>
@@ -1866,10 +1875,10 @@
       </c>
       <c r="B43" s="11"/>
       <c r="C43" s="12" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="180.6" customHeight="1">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="180.65" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>52</v>
       </c>
@@ -1877,7 +1886,7 @@
         <v>148</v>
       </c>
       <c r="C44" s="35" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D44" s="30"/>
     </row>
@@ -1905,7 +1914,7 @@
         <v>56</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="14.25" customHeight="1">
@@ -1922,7 +1931,7 @@
         <v>59</v>
       </c>
       <c r="C50" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D50" s="4"/>
     </row>
@@ -1934,7 +1943,7 @@
         <v>61</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D51" s="4"/>
     </row>
@@ -1943,7 +1952,7 @@
         <v>62</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D52" s="4"/>
     </row>
@@ -1974,7 +1983,7 @@
         <v>67</v>
       </c>
       <c r="C55" s="32" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D55" s="4"/>
     </row>
@@ -1986,7 +1995,7 @@
         <v>69</v>
       </c>
       <c r="C56" s="32" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D56" s="4"/>
     </row>
@@ -1998,7 +2007,7 @@
         <v>70</v>
       </c>
       <c r="C57" s="32" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D57" s="4"/>
     </row>
@@ -2010,7 +2019,7 @@
         <v>71</v>
       </c>
       <c r="C58" s="32" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D58" s="4"/>
     </row>
@@ -2022,11 +2031,11 @@
         <v>73</v>
       </c>
       <c r="C59" s="32" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D59" s="4"/>
     </row>
-    <row r="60" spans="1:4" ht="60.75" thickBot="1">
+    <row r="60" spans="1:4" ht="58.5" thickBot="1">
       <c r="A60" s="15" t="s">
         <v>74</v>
       </c>
@@ -2034,11 +2043,11 @@
         <v>75</v>
       </c>
       <c r="C60" s="32" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D60" s="4"/>
     </row>
-    <row r="61" spans="1:4" ht="15.75" thickBot="1">
+    <row r="61" spans="1:4" thickBot="1">
       <c r="A61" s="15" t="s">
         <v>164</v>
       </c>
@@ -2046,7 +2055,7 @@
         <v>76</v>
       </c>
       <c r="C61" s="32" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D61" s="4"/>
     </row>
@@ -2058,7 +2067,7 @@
         <v>78</v>
       </c>
       <c r="C62" s="32" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D62" s="4"/>
     </row>
@@ -2070,7 +2079,7 @@
         <v>79</v>
       </c>
       <c r="C63" s="33" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D63" s="4"/>
     </row>
@@ -2082,7 +2091,7 @@
         <v>81</v>
       </c>
       <c r="C64" s="32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D64" s="4"/>
     </row>
@@ -2094,7 +2103,7 @@
         <v>83</v>
       </c>
       <c r="C65" s="32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D65" s="4"/>
     </row>
@@ -2106,7 +2115,7 @@
         <v>85</v>
       </c>
       <c r="C66" s="32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D66" s="4"/>
     </row>
@@ -2116,7 +2125,7 @@
       </c>
       <c r="B67" s="15"/>
       <c r="C67" s="32" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D67" s="4"/>
     </row>
@@ -2128,7 +2137,7 @@
         <v>88</v>
       </c>
       <c r="C68" s="33" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D68" s="4"/>
     </row>
@@ -2140,7 +2149,7 @@
         <v>90</v>
       </c>
       <c r="C69" s="32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D69" s="4"/>
     </row>
@@ -2152,7 +2161,7 @@
         <v>92</v>
       </c>
       <c r="C70" s="32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D70" s="4"/>
     </row>
@@ -2164,7 +2173,7 @@
         <v>94</v>
       </c>
       <c r="C71" s="32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D71" s="4"/>
     </row>
@@ -2176,7 +2185,7 @@
         <v>98</v>
       </c>
       <c r="C72" s="32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D72" s="4"/>
     </row>
@@ -2198,7 +2207,7 @@
         <v>169</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="14.25" customHeight="1" thickBot="1">
@@ -2210,7 +2219,7 @@
       </c>
       <c r="C75" s="32"/>
     </row>
-    <row r="76" spans="1:4" ht="14.45" customHeight="1" thickBot="1">
+    <row r="76" spans="1:4" ht="14.5" customHeight="1" thickBot="1">
       <c r="A76" s="15" t="s">
         <v>170</v>
       </c>
@@ -2219,7 +2228,7 @@
       </c>
       <c r="C76" s="32"/>
     </row>
-    <row r="77" spans="1:4" ht="14.45" customHeight="1" thickBot="1">
+    <row r="77" spans="1:4" ht="14.5" customHeight="1" thickBot="1">
       <c r="A77" s="19" t="s">
         <v>95</v>
       </c>
@@ -2227,7 +2236,7 @@
         <v>96</v>
       </c>
       <c r="C77" s="31" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="14.25" customHeight="1" thickBot="1">
@@ -2247,10 +2256,10 @@
       </c>
       <c r="B80" s="2"/>
       <c r="C80" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="44.1" customHeight="1">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="44.15" customHeight="1">
       <c r="C81" s="3"/>
     </row>
     <row r="82" spans="1:3" ht="51" customHeight="1">
@@ -2274,19 +2283,20 @@
     </row>
     <row r="85" spans="1:3" ht="14.25" customHeight="1">
       <c r="A85" s="38" t="s">
+        <v>230</v>
+      </c>
+      <c r="B85" s="39" t="s">
         <v>231</v>
       </c>
-      <c r="B85" s="39" t="s">
-        <v>232</v>
-      </c>
       <c r="C85" s="39"/>
     </row>
-    <row r="86" spans="1:3" ht="51.6" customHeight="1">
+    <row r="86" spans="1:3" ht="51.65" customHeight="1">
       <c r="A86" s="40" t="s">
-        <v>220</v>
-      </c>
-      <c r="B86" s="41" t="s">
-        <v>173</v>
+        <v>219</v>
+      </c>
+      <c r="B86" s="41" t="str">
+        <f>_xlfn.CONCAT(E4,  ":\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json")</f>
+        <v>D:\Procesos_UiPath\Llaves\crp-pro-ccoe-automat-c9c501f57fdd_NF.json</v>
       </c>
       <c r="C86" s="42" t="s">
         <v>124</v>
@@ -2294,16 +2304,16 @@
     </row>
     <row r="87" spans="1:3" ht="42" customHeight="1">
       <c r="A87" s="40" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B87" s="43" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C87" s="42" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="14.1" customHeight="1">
+    <row r="88" spans="1:3" ht="14.15" customHeight="1">
       <c r="A88" s="2" t="s">
         <v>103</v>
       </c>
@@ -3247,12 +3257,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z996"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
-    <col min="2" max="2" width="89.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="92.5703125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="89.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="92.54296875" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -3297,7 +3307,7 @@
         <v>20</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -3331,7 +3341,7 @@
         <v>126</v>
       </c>
       <c r="C3" s="44" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -3385,7 +3395,7 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" ht="30">
+    <row r="5" spans="1:26" ht="29">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -3396,7 +3406,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="30">
+    <row r="6" spans="1:26" ht="29">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -3407,12 +3417,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:26" ht="14.5">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="6"/>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" spans="1:26" ht="14.5">
       <c r="A8" t="s">
         <v>117</v>
       </c>
@@ -3420,10 +3430,10 @@
         <v>122</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.5">
       <c r="A9" t="s">
         <v>118</v>
       </c>
@@ -3431,10 +3441,10 @@
         <v>465</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.5">
       <c r="A10" t="s">
         <v>119</v>
       </c>
@@ -3442,10 +3452,10 @@
         <v>121</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.5">
       <c r="A11" t="s">
         <v>120</v>
       </c>
@@ -3453,74 +3463,74 @@
         <v>993</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.5">
       <c r="A12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B12" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="B12" s="21" t="s">
-        <v>201</v>
-      </c>
       <c r="C12" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.5">
       <c r="A13" t="s">
         <v>126</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="14.5">
       <c r="A14" s="45" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="B14" s="49" t="s">
+      <c r="C14" s="46" t="s">
         <v>203</v>
-      </c>
-      <c r="C14" s="46" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="B15" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="B15" s="50" t="s">
+      <c r="C15" s="46" t="s">
         <v>206</v>
-      </c>
-      <c r="C15" s="46" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" s="50" t="s">
         <v>208</v>
       </c>
-      <c r="B16" s="50" t="s">
+      <c r="C16" s="46" t="s">
         <v>209</v>
-      </c>
-      <c r="C16" s="46" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" s="45" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B17" s="50" t="str">
         <f>"D:\Procesos_UiPath\"&amp;Settings!B3&amp;"\"</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
@@ -3531,7 +3541,7 @@
         <v>42</v>
       </c>
       <c r="B19" s="8" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;Settings!B3&amp;"\Archivos"</f>
+        <f>_xlfn.CONCAT(Settings!E4,":\Procesos_UiPath\"&amp;Settings!B3&amp;"\Archivos")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos</v>
       </c>
       <c r="C19" s="8" t="s">
@@ -3543,7 +3553,7 @@
         <v>6</v>
       </c>
       <c r="B20" s="21" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;Settings!B3&amp;"\Archivos\Exceptions_Screenshots"</f>
+        <f>_xlfn.CONCAT(Settings!E4, ":\Procesos_UiPath\"&amp;Settings!B3&amp;"\Archivos\Exceptions_Screenshots")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\Exceptions_Screenshots</v>
       </c>
       <c r="C20" t="s">
@@ -3605,7 +3615,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" ht="14.5">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -3651,10 +3661,10 @@
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" s="23" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B30" s="47" t="str">
-        <f>"D:\Procesos_UiPath\"&amp;Settings!B3&amp;"\Archivos\LOG"</f>
+        <f>_xlfn.CONCAT(Settings!E4,":\Procesos_UiPath\"&amp;Settings!B3&amp;"\Archivos\LOG")</f>
         <v>D:\Procesos_UiPath\340_CUADREAJUSTESMONE_NF_FNF_CCRE\Archivos\LOG</v>
       </c>
     </row>
@@ -4633,12 +4643,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" customWidth="1"/>
+    <col min="2" max="2" width="30.1796875" customWidth="1"/>
+    <col min="3" max="3" width="60.26953125" customWidth="1"/>
+    <col min="4" max="26" width="65.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -5685,15 +5695,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="65.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="65.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75">
+    <row r="1" spans="1:4" ht="18.5">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -5709,13 +5719,13 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D2" t="s">
         <v>45</v>
@@ -5723,16 +5733,16 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B3" t="s">
         <v>228</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D3" t="s">
         <v>229</v>
-      </c>
-      <c r="C3" t="s">
-        <v>223</v>
-      </c>
-      <c r="D3" t="s">
-        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>